<commit_message>
feat: sheet4의 DEFENSE_DESIGNATION_DATE도 NULL로 나오게 수정
</commit_message>
<xml_diff>
--- a/src/main/resources/excel/exceldata.xlsx
+++ b/src/main/resources/excel/exceldata.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1171" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1411" uniqueCount="291">
   <si>
     <t>company_id</t>
   </si>
@@ -926,6 +926,24 @@
   </si>
   <si>
     <t>26.02.25</t>
+  </si>
+  <si>
+    <t>2026-02-25 13:46:34</t>
+  </si>
+  <si>
+    <t>2026-02-25 13:47:04</t>
+  </si>
+  <si>
+    <t>2026-02-25 13:51:51</t>
+  </si>
+  <si>
+    <t>2026-02-25 13:52:18</t>
+  </si>
+  <si>
+    <t>NULL</t>
+  </si>
+  <si>
+    <t>2026-02-25 13:55:22</t>
   </si>
 </sst>
 </file>
@@ -2952,7 +2970,7 @@
     <col min="6" max="6" bestFit="true" customWidth="true" width="10.0"/>
     <col min="7" max="7" bestFit="true" customWidth="true" width="13.0"/>
     <col min="8" max="8" bestFit="true" customWidth="true" width="14.40234375"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="15.0"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="18.23046875"/>
     <col min="10" max="10" bestFit="true" customWidth="true" width="13.0"/>
     <col min="11" max="11" bestFit="true" customWidth="true" width="13.0"/>
     <col min="12" max="12" bestFit="true" customWidth="true" width="15.0"/>
@@ -3010,7 +3028,7 @@
         <v>127</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="F2" t="s" s="0">
         <v>98</v>
@@ -3022,7 +3040,7 @@
         <v>174</v>
       </c>
       <c r="I2" t="s" s="0">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="J2" t="s" s="0">
         <v>80</v>
@@ -3048,7 +3066,7 @@
         <v>127</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="F3" t="s" s="0">
         <v>98</v>
@@ -3060,7 +3078,7 @@
         <v>174</v>
       </c>
       <c r="I3" t="s" s="0">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="J3" t="s" s="0">
         <v>80</v>
@@ -3086,7 +3104,7 @@
         <v>127</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="F4" t="s" s="0">
         <v>98</v>
@@ -3098,7 +3116,7 @@
         <v>174</v>
       </c>
       <c r="I4" t="s" s="0">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="J4" t="s" s="0">
         <v>80</v>

</xml_diff>

<commit_message>
feat: sheet4의 UPDATE_ID,IP,DATE 부분 \N에서 NULL로 변경
</commit_message>
<xml_diff>
--- a/src/main/resources/excel/exceldata.xlsx
+++ b/src/main/resources/excel/exceldata.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1411" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1459" uniqueCount="292">
   <si>
     <t>company_id</t>
   </si>
@@ -944,6 +944,9 @@
   </si>
   <si>
     <t>2026-02-25 13:55:22</t>
+  </si>
+  <si>
+    <t>2026-02-25 14:07:48</t>
   </si>
 </sst>
 </file>
@@ -3040,16 +3043,16 @@
         <v>174</v>
       </c>
       <c r="I2" t="s" s="0">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="J2" t="s" s="0">
-        <v>80</v>
+        <v>289</v>
       </c>
       <c r="K2" t="s" s="0">
-        <v>80</v>
+        <v>289</v>
       </c>
       <c r="L2" t="s" s="0">
-        <v>80</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3">
@@ -3078,16 +3081,16 @@
         <v>174</v>
       </c>
       <c r="I3" t="s" s="0">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="J3" t="s" s="0">
-        <v>80</v>
+        <v>289</v>
       </c>
       <c r="K3" t="s" s="0">
-        <v>80</v>
+        <v>289</v>
       </c>
       <c r="L3" t="s" s="0">
-        <v>80</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4">
@@ -3116,16 +3119,16 @@
         <v>174</v>
       </c>
       <c r="I4" t="s" s="0">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="J4" t="s" s="0">
-        <v>80</v>
+        <v>289</v>
       </c>
       <c r="K4" t="s" s="0">
-        <v>80</v>
+        <v>289</v>
       </c>
       <c r="L4" t="s" s="0">
-        <v>80</v>
+        <v>289</v>
       </c>
     </row>
   </sheetData>

</xml_diff>